<commit_message>
Weekly sales report update
</commit_message>
<xml_diff>
--- a/outputs/Sales_Reporting_2026.xlsx
+++ b/outputs/Sales_Reporting_2026.xlsx
@@ -803,7 +803,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -896,7 +896,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tempo k cíli – kumulativní Won vs. Goal</a:t>
+              <a:t>Tempo k cíli – Won vs. Goal</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1613,7 +1613,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1706,7 +1706,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tempo k cíli – kumulativní Won vs. Goal</a:t>
+              <a:t>Tempo k cíli – Won vs. Goal</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -2287,7 +2287,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -2380,7 +2380,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tempo k cíli – kumulativní Won vs. Goal</a:t>
+              <a:t>Tempo k cíli – Won vs. Goal</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -2724,7 +2724,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3054,7 +3054,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3147,7 +3147,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tempo k cíli – kumulativní Won vs. Goal</a:t>
+              <a:t>Tempo k cíli – Won vs. Goal</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3728,7 +3728,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3925,7 +3925,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tempo k cíli – kumulativní Won vs. Goal</a:t>
+              <a:t>Tempo k cíli – Won vs. Goal</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -4402,7 +4402,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -4940,7 +4940,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -5033,7 +5033,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tempo k cíli – kumulativní Won vs. Goal</a:t>
+              <a:t>Tempo k cíli – Won vs. Goal</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -5905,7 +5905,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Funnel – rozpad pipeline podle stage (06.07.)</a:t>
+              <a:t>Funnel – rozpad pipeline (12.07.)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -7485,7 +7485,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generováno týdně z HubSpotu (nahrazuje ruční doplňování)</t>
+          <t>Generováno týdně z HubSpotu</t>
         </is>
       </c>
     </row>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -9861,7 +9861,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -11001,7 +11001,7 @@
         <v>3610753</v>
       </c>
       <c r="U22" s="14" t="n">
-        <v>4087400</v>
+        <v>4134600</v>
       </c>
     </row>
     <row r="23">
@@ -11387,7 +11387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G784"/>
+  <dimension ref="A1:G795"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11409,7 +11409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generováno týdně z HubSpotu (nahrazuje ruční doplňování)</t>
+          <t>Generováno týdně z HubSpotu</t>
         </is>
       </c>
     </row>
@@ -32126,16 +32126,16 @@
     </row>
     <row r="779">
       <c r="A779" s="4" t="n">
-        <v>396380044523</v>
+        <v>16200551119</v>
       </c>
       <c r="B779" s="4" t="inlineStr">
         <is>
-          <t>Mashreq Pakistan, Seamless Rijad 25</t>
+          <t>Jordan Ahli Bank, woodpecker</t>
         </is>
       </c>
       <c r="C779" s="4" t="inlineStr">
         <is>
-          <t>Mashreq</t>
+          <t>Jordan Ahli Bank</t>
         </is>
       </c>
       <c r="D779" s="4" t="inlineStr">
@@ -32147,22 +32147,22 @@
         <v>46219</v>
       </c>
       <c r="F779" s="6" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="G779" s="4" t="inlineStr"/>
     </row>
     <row r="780">
       <c r="A780" s="4" t="n">
-        <v>460476222664</v>
+        <v>245212643546</v>
       </c>
       <c r="B780" s="4" t="inlineStr">
         <is>
-          <t>Al Barid Bank - from HPS</t>
+          <t>Fintech Dubai:Wio UAE</t>
         </is>
       </c>
       <c r="C780" s="4" t="inlineStr">
         <is>
-          <t>Al Barid Bank</t>
+          <t>Wio UAE</t>
         </is>
       </c>
       <c r="D780" s="4" t="inlineStr">
@@ -32174,22 +32174,22 @@
         <v>46219</v>
       </c>
       <c r="F780" s="6" t="n">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="G780" s="4" t="inlineStr"/>
     </row>
     <row r="781">
       <c r="A781" s="4" t="n">
-        <v>501313743042</v>
+        <v>285342572762</v>
       </c>
       <c r="B781" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank DXB - discovery</t>
+          <t>Source: Linkedin; Company: Banque Patronus</t>
         </is>
       </c>
       <c r="C781" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Banque Patronus</t>
         </is>
       </c>
       <c r="D781" s="4" t="inlineStr">
@@ -32201,22 +32201,22 @@
         <v>46219</v>
       </c>
       <c r="F781" s="6" t="n">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="G781" s="4" t="inlineStr"/>
     </row>
     <row r="782">
       <c r="A782" s="4" t="n">
-        <v>501500277973</v>
+        <v>495269111005</v>
       </c>
       <c r="B782" s="4" t="inlineStr">
         <is>
-          <t>HSBC - Dubai OH</t>
+          <t>Manager.one: Melanie FAUCHON - contact form</t>
         </is>
       </c>
       <c r="C782" s="4" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>Manager.one</t>
         </is>
       </c>
       <c r="D782" s="4" t="inlineStr">
@@ -32228,22 +32228,22 @@
         <v>46219</v>
       </c>
       <c r="F782" s="6" t="n">
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="G782" s="4" t="inlineStr"/>
     </row>
     <row r="783">
       <c r="A783" s="4" t="n">
-        <v>501500997841</v>
+        <v>285715078373</v>
       </c>
       <c r="B783" s="4" t="inlineStr">
         <is>
-          <t>Abacus Pakistan - OH LinkedIn</t>
+          <t>AXIS India</t>
         </is>
       </c>
       <c r="C783" s="4" t="inlineStr">
         <is>
-          <t>Abacus Cambridge Partners</t>
+          <t>Axis Bank</t>
         </is>
       </c>
       <c r="D783" s="4" t="inlineStr">
@@ -32255,22 +32255,22 @@
         <v>46219</v>
       </c>
       <c r="F783" s="6" t="n">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="G783" s="4" t="inlineStr"/>
     </row>
     <row r="784">
       <c r="A784" s="4" t="n">
-        <v>496001859797</v>
+        <v>311526355159</v>
       </c>
       <c r="B784" s="4" t="inlineStr">
         <is>
-          <t>Moved to Tapix: Inbound - Manager.one - New Deal</t>
+          <t>MoneyKSA: BSF</t>
         </is>
       </c>
       <c r="C784" s="4" t="inlineStr">
         <is>
-          <t>Manager.one</t>
+          <t>Banque Saudi Fransi</t>
         </is>
       </c>
       <c r="D784" s="4" t="inlineStr">
@@ -32282,9 +32282,306 @@
         <v>46219</v>
       </c>
       <c r="F784" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G784" s="4" t="inlineStr"/>
+    </row>
+    <row r="785">
+      <c r="A785" s="4" t="n">
+        <v>311549636806</v>
+      </c>
+      <c r="B785" s="4" t="inlineStr">
+        <is>
+          <t>MoneyKSA: Drahim</t>
+        </is>
+      </c>
+      <c r="C785" s="4" t="inlineStr">
+        <is>
+          <t>Drahim</t>
+        </is>
+      </c>
+      <c r="D785" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E785" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F785" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G785" s="4" t="inlineStr"/>
+    </row>
+    <row r="786">
+      <c r="A786" s="4" t="n">
+        <v>311146490054</v>
+      </c>
+      <c r="B786" s="4" t="inlineStr">
+        <is>
+          <t>MoneyKSA: D360 Bank</t>
+        </is>
+      </c>
+      <c r="C786" s="4" t="inlineStr">
+        <is>
+          <t>D360 Bank</t>
+        </is>
+      </c>
+      <c r="D786" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E786" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F786" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G786" s="4" t="inlineStr"/>
+    </row>
+    <row r="787">
+      <c r="A787" s="4" t="n">
+        <v>311146494155</v>
+      </c>
+      <c r="B787" s="4" t="inlineStr">
+        <is>
+          <t>LiP2025: United Arab Bank</t>
+        </is>
+      </c>
+      <c r="C787" s="4" t="inlineStr">
+        <is>
+          <t>United Arab Bank</t>
+        </is>
+      </c>
+      <c r="D787" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E787" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F787" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G787" s="4" t="inlineStr"/>
+    </row>
+    <row r="788">
+      <c r="A788" s="4" t="n">
+        <v>375461881079</v>
+      </c>
+      <c r="B788" s="4" t="inlineStr">
+        <is>
+          <t>Source: SFF25; Company: Mashreq</t>
+        </is>
+      </c>
+      <c r="C788" s="4" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="D788" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E788" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F788" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G788" s="4" t="inlineStr"/>
+    </row>
+    <row r="789">
+      <c r="A789" s="4" t="n">
+        <v>360458783986</v>
+      </c>
+      <c r="B789" s="4" t="inlineStr">
+        <is>
+          <t>ATM Nearby: Axis Bank - New Deal (Tapix)</t>
+        </is>
+      </c>
+      <c r="C789" s="4" t="inlineStr">
+        <is>
+          <t>Axis Bank</t>
+        </is>
+      </c>
+      <c r="D789" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E789" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F789" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G789" s="4" t="inlineStr"/>
+    </row>
+    <row r="790">
+      <c r="A790" s="4" t="n">
+        <v>396380044523</v>
+      </c>
+      <c r="B790" s="4" t="inlineStr">
+        <is>
+          <t>Mashreq Pakistan, Seamless Rijad 25</t>
+        </is>
+      </c>
+      <c r="C790" s="4" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="D790" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E790" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F790" s="6" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G790" s="4" t="inlineStr"/>
+    </row>
+    <row r="791">
+      <c r="A791" s="4" t="n">
+        <v>460476222664</v>
+      </c>
+      <c r="B791" s="4" t="inlineStr">
+        <is>
+          <t>Al Barid Bank - from HPS</t>
+        </is>
+      </c>
+      <c r="C791" s="4" t="inlineStr">
+        <is>
+          <t>Al Barid Bank</t>
+        </is>
+      </c>
+      <c r="D791" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E791" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F791" s="6" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G791" s="4" t="inlineStr"/>
+    </row>
+    <row r="792">
+      <c r="A792" s="4" t="n">
+        <v>501313743042</v>
+      </c>
+      <c r="B792" s="4" t="inlineStr">
+        <is>
+          <t>Standard Chartered Bank DXB - discovery</t>
+        </is>
+      </c>
+      <c r="C792" s="4" t="inlineStr">
+        <is>
+          <t>Standard Chartered Bank</t>
+        </is>
+      </c>
+      <c r="D792" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E792" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F792" s="6" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G792" s="4" t="inlineStr"/>
+    </row>
+    <row r="793">
+      <c r="A793" s="4" t="n">
+        <v>501500277973</v>
+      </c>
+      <c r="B793" s="4" t="inlineStr">
+        <is>
+          <t>HSBC - Dubai OH</t>
+        </is>
+      </c>
+      <c r="C793" s="4" t="inlineStr">
+        <is>
+          <t>HSBC</t>
+        </is>
+      </c>
+      <c r="D793" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E793" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F793" s="6" t="n">
+        <v>150000</v>
+      </c>
+      <c r="G793" s="4" t="inlineStr"/>
+    </row>
+    <row r="794">
+      <c r="A794" s="4" t="n">
+        <v>501500997841</v>
+      </c>
+      <c r="B794" s="4" t="inlineStr">
+        <is>
+          <t>Abacus Pakistan - OH LinkedIn</t>
+        </is>
+      </c>
+      <c r="C794" s="4" t="inlineStr">
+        <is>
+          <t>Abacus Cambridge Partners</t>
+        </is>
+      </c>
+      <c r="D794" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E794" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F794" s="6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G794" s="4" t="inlineStr"/>
+    </row>
+    <row r="795">
+      <c r="A795" s="4" t="n">
+        <v>496001859797</v>
+      </c>
+      <c r="B795" s="4" t="inlineStr">
+        <is>
+          <t>Moved to Tapix: Inbound - Manager.one - New Deal</t>
+        </is>
+      </c>
+      <c r="C795" s="4" t="inlineStr">
+        <is>
+          <t>Manager.one</t>
+        </is>
+      </c>
+      <c r="D795" s="4" t="inlineStr">
+        <is>
+          <t>Olda</t>
+        </is>
+      </c>
+      <c r="E795" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F795" s="6" t="n">
         <v>34175</v>
       </c>
-      <c r="G784" s="4" t="inlineStr"/>
+      <c r="G795" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -32444,7 +32741,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -34014,7 +34311,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -35517,7 +35814,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -37087,7 +37384,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -38657,7 +38954,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -40227,7 +40524,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>
@@ -41367,7 +41664,7 @@
         <v>164500</v>
       </c>
       <c r="U22" s="14" t="n">
-        <v>181500</v>
+        <v>228700</v>
       </c>
     </row>
     <row r="23">
@@ -41797,7 +42094,7 @@
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
-          <t>06.07.</t>
+          <t>12.07.</t>
         </is>
       </c>
     </row>

</xml_diff>